<commit_message>
Bieroverzicht bijgewerkt 13-09-2026 20:17
</commit_message>
<xml_diff>
--- a/docs/bieroverzicht.xlsx
+++ b/docs/bieroverzicht.xlsx
@@ -33489,7 +33489,7 @@
         <v>4.11</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>2108</v>
+        <v>2135</v>
       </c>
       <c r="F5" s="5" t="n">
         <v>7.95</v>
@@ -33602,7 +33602,7 @@
         <v>4.24</v>
       </c>
       <c r="E8" s="2" t="n">
-        <v>1067</v>
+        <v>1090</v>
       </c>
       <c r="F8" s="5" t="n">
         <v>6.95</v>
@@ -33639,7 +33639,7 @@
         <v>4.24</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>1289</v>
+        <v>1296</v>
       </c>
       <c r="F9" s="5" t="n">
         <v>7.5</v>
@@ -33676,7 +33676,7 @@
         <v>4.18</v>
       </c>
       <c r="E10" s="2" t="n">
-        <v>1368</v>
+        <v>1375</v>
       </c>
       <c r="F10" s="5" t="n">
         <v>6.95</v>
@@ -34013,7 +34013,7 @@
         <v>4.09</v>
       </c>
       <c r="E19" s="2" t="n">
-        <v>1788</v>
+        <v>1793</v>
       </c>
       <c r="F19" s="5" t="n">
         <v>6.95</v>
@@ -34050,7 +34050,7 @@
         <v>4.04</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>59412</v>
+        <v>59454</v>
       </c>
       <c r="F20" s="5" t="n">
         <v>7.95</v>

</xml_diff>